<commit_message>
Agrega direcciones, actividad y subsector textil a los prospectos
34 prospectos A/B con dirección publicada (32 encontradas), giro y
subsector; columnas nuevas en el Excel interno.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012axCVDM5kAgj1VFnxhpsuM
</commit_message>
<xml_diff>
--- a/propuesta-clt/Prospectos_CLT_Mexico_INTERNO.xlsx
+++ b/propuesta-clt/Prospectos_CLT_Mexico_INTERNO.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospectos'!$A$1:$M$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospectos'!$A$1:$Q$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,22 +446,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,45 +491,65 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Dirección publicada</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>A qué se dedica</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Subsector textil</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Dirección verificada</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Por qué es prospecto</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Sitio web</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Contacto publicado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Estatus</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Próximo paso</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -554,33 +578,53 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>12 de Octubre No. 805, Col. Industrial Alce Blanco, C.P. 53370, Naucalpan de Juárez, Estado de México</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Maquila industrial de serigrafía textil de alto volumen (más de 130,000 piezas/semana) para marcas, retailers y licencias, con producción apta para EE.UU. y Canadá.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Maquila industrial con carrusel automático, hasta 18 tintas, +130,000 piezas/semana, tintas ECO PASSPORT y producción para USA/Canadá. Candidato ideal para estaciones digitales y tintas especiales.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>https://adnserigrafia.com.mx/</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://adnserigrafia.com.mx/</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -605,33 +649,53 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Blvd. Centro Industrial No. 24, Col. Industrial Puente de Vigas, Tlalnepantla, Estado de México</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Diseña, confecciona y decora (serigrafía y bordado) prendas como playeras, sudaderas, pants, pijamas y gorras para marcas.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Maquila de exportación de confección (IMMEX, SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Diseña, confecciona y decora prendas desde 1986; maquila auditada (SMETA, Inditex, C&amp;A); serigrafía y bordado propios; marca JHK.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>https://clabeck.com/</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-playeras-en-mexico.php</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -656,33 +720,53 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Cto. Dr. Gustavo Baz 5-A, México Nuevo, C.P. 52966, Cd. López Mateos (Atizapán de Zaragoza), Estado de México</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Empresa textil verticalmente integrada (Zentrix Industrial Mexico) que produce telas sintéticas y fabrica ropa deportiva (activewear) y lencería para marcas.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Maquila de exportación de confección (IMMEX, SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Manufactura de paquete completo para marcas globales (se mencionan Nike/Lululemon). Volumen alto; posible decoración interna (por confirmar).</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>https://zentrix.com.mx/</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -707,33 +791,53 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>Av. Dr. Mateo del Regil 6, El Briseño, C.P. 45236, Zapopan, Jalisco (showroom según directorio; la planta está en Puente Grande, Jal., sin calle publicada)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Fabrica y distribuye playeras básicas, deportivas (Dry-Fit) y promocionales (marca Mindy) en una planta automatizada de 5,000 m² en Puente Grande, Jalisco.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Fábrica de playeras deportivas y publicitarias de gran escala; nave automatizada de 5,000 m²; atiende exportación a EE.UU.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>https://www.grupodiermi.com/</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-playeras-en-mexico.php</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr"/>
+      <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -758,29 +862,49 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>Priv. San Isidro s/n, Barrio San Isidro, Santa María Zacatepec, Juan C. Bonilla, Puebla, C.P. 72660</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Maquila de confección en tejido de punto y plano para marcas (250 máquinas de costura), con programa IMMEX y auditorías de Target, Sears, Kohl's y Macy's.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Maquila de exportación de confección (IMMEX, SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Maquila de playera tubular para marcas, con capacidad de 80,000 piezas/semana en corte y 60,000 en costura; el directorio menciona estampado serigráfico.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/proveedores-de-ropa-directo-de-fabrica-en-puebla.html</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -805,37 +929,57 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Privada Nuevo León 406, Colonia El Carmen, C.P. 72530, Puebla, Pue.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Serigrafía textil automatizada por volumen de playeras para campañas, eventos deportivos y promocionales.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Serigrafía textil automatizada por volumen (playeras de campaña política, deportivas, promocionales) con más de 30 años. Perfil ideal para un híbrido.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>https://serigrafiatextil.com.mx/</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>(222) 682 0694</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://serigrafiatextil.com.mx/</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -860,33 +1004,53 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>Cerro de la Silla No. 3011, Colonia 15 de Mayo, Guadalupe, N.L., C.P. 67177 (también: Nube 3, Ampliación Santa Catarina, Valle de Chalco Solidaridad, Edo. de México, C.P. 56610)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Fábrica integrada de playeras promocionales y para campañas de alto volumen con serigrafía de hasta 12 colores.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Promocionales y prendas publicitarias</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
           <t>Promocionales</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Fábrica integrada (hilo a prenda) con más de 30 años, especializada en playeras para campañas políticas y publicitarias de alto volumen.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>https://reitex.mx/</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-playeras-en-mexico.php</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -911,29 +1075,49 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>C. 20 131-C, Centro, C.P. 97450, Baca, Yucatán</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Fabricante verticalmente integrado de telas de punto y prendas premium para marcas internacionales, con 7 sitios de producción (Puebla, Baca, Tizimín, Peto, Espita y Campeche).</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Tejido de punto y confección (SCIAN 3132/315)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Uno de los mayores productores de tejido de punto del país (más de 16-25 millones de prendas/año) con serigrafía y bordado internos; clientes Nike, Fanatics, Tommy Hilfiger, Patagonia.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://mexicoindustry.com/noticia/vertical-knits-inicia-construccion-de-su-planta-en-yucatan</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr"/>
+      <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -958,29 +1142,53 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>Venustiano Carranza número 91, Colonia Centro, Alcaldía Cuauhtémoc, C.P. 06060, Ciudad de México (domicilio publicado en su aviso de privacidad)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Marca y cadena mexicana de ropa de moda con tiendas propias y venta en línea.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Marca de moda / diseño</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
           <t>Marca de moda</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Marca mexicana de moda (desde 2007) con gráficos estampados; contrata personal de estampado (serigrafía, rotativa, digital). Interesa para efectos especiales (silicón 3D) y digital.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>https://mx.indeed.com/q-de-estampados-para-l-naucalpan,-m%C3%A9x.-empleos.html</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>https://mx.indeed.com/q-de-estampados-para-l-naucalpan,-m%C3%A9x.-empleos.html</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>El domicilio publicado está en CDMX (Centro), no en Naucalpan; es principalmente retailer y no se confirmó en su sitio que estampe en planta propia.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1005,33 +1213,53 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
+          <t>Juan Hernández y Dávalos 61 PB, Col. Algarín, Alcaldía Cuauhtémoc, C.P. 06880, Ciudad de México (matriz)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica y distribuye playeras, sudaderas y textiles promocionales personalizados para empresas, eventos y campañas publicitarias.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Promocionales y prendas publicitarias</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
           <t>Promocionales</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Fábrica de playeras y sudaderas con más de 25 años; producción a gran escala para campañas y empresas, con serigrafía, sublimación y bordado propios.</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>https://www.gocas.com.mx/</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-sudaderas-en-mexico.php</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1056,33 +1284,53 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
+          <t>C. Hormona 11, C.P. 53500, Naucalpan de Juárez, Estado de México</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Grupo de manufactura textil deportiva que produce prendas de alto rendimiento para marcas como Adidas, Puma y Charly.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Fabricante textil de gran volumen; según el directorio, hace uniformes oficiales FIFA. Buen perfil para estampado de alto volumen.</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>https://grupomartex.com/</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1107,33 +1355,53 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
+          <t>Calle 3 #4, Alce Blanco, Naucalpan, Estado de México, C.P. 53370</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica prendas multiestilo y desarrolla y comercializa tejidos y confecciones para clientes nacionales e internacionales.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Confección de prendas de vestir (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>Paquete completo y marca privada (private label) para mercado nacional e internacional.</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>https://www.karabe.com.mx/</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-mexico.html</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1158,33 +1426,53 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
+          <t>Tlacotal B 2309, Ciudad de México (colonia y C.P. no publicados en el sitio)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Taller de maquila serigráfica por volumen (plastisol, base agua y corrosión) para fábricas, talleres y marcas; también DTF y sublimación.</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>Taller de maquila serigráfica con más de 20 años; produce por volumen en plastisol, base agua y corrosión para fábricas y marcas; también DTF y sublimación.</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>https://serigrafiartesp.com/</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>https://serigrafiartesp.com/</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr"/>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1209,29 +1497,53 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>No publicada</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Marca jalisciense de ropa y uniformes deportivos (Deportextiles, S.A. de C.V., fundada en 1994, sede en Zapopan según Wikipedia); su tienda en línea está cerrada con contraseña en espera de relanzamiento.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Marca jalisciense de ropa deportiva que vistió a clubes de Liga MX; produce jerseys y uniformes de equipo. Su tamaño actual está por verificar.</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.merca20.com/?p=133184</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.merca20.com/?p=133184</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr"/>
+      <c r="P15" s="3" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Sitio atletica.com cerrado con contraseña ('próximamente'); marca en relanzamiento, capacidad productiva actual no confirmada.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1256,29 +1568,49 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
+          <t>Eliseo Granja #3, Col. Revolucionaria, Guadalajara, Jalisco (C.P. 44960 según directorio)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica uniformes escolares, empresariales y deportivos con bordado, impresión DTF y tejido de cuellos y puños.</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Uniformes escolares, empresariales y deportivos con bordado y DTF; atiende pedidos masivos. Podría pasar de DTF a un híbrido.</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-guadalajara-jalisco.html</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-guadalajara-jalisco.html</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1303,33 +1635,53 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
+          <t>Leandro Valle 1159, Centro, Guadalajara, Jalisco</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Taller de serigrafía textil de playeras, uniformes y promocionales en Guadalajara, con más de 15 años de experiencia.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Serigrafía textil de uniformes y promocionales, y maquila para marcas de moda en Guadalajara.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>https://neurographics.com.mx/</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>https://neurographics.com.mx/serigrafia-en-guadalajara/</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr"/>
+      <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1354,33 +1706,53 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
+          <t>Av. Pablo Neruda 4341, Local G1, Jardines Universidad, C.P. 45110, Zapopan, Jalisco</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Crea, produce y comercializa ropa, accesorios y uniformes deportivos personalizados para equipos.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Uniformes deportivos personalizados para equipos, con red de distribuidores; buen candidato para estaciones digitales (nombres y números variables).</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>https://romed.com.mx/</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr"/>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1405,33 +1777,53 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>Av. Enrique Díaz de León Sur 761, Col. Moderna, Guadalajara, Jalisco, C.P. 44190</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica uniformes industriales y ropa de trabajo (playeras, camisas, batas, overoles) con servicios de bordado y estampado.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>Fabricante de uniformes con más de 30 años; ofrece serigrafía, bordado y transfer, y anuncia maquila de estampado por alto volumen.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>https://uniformescarmen.com.mx/</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>https://uniformescarmen.com.mx/estampado-de-playeras-cerca-de-zapopan-jalisco/</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr"/>
+      <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1456,29 +1848,49 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>Boulevard Cholula-Huejotzingo No. 727, San Sebastián Tepalcatepec, San Pedro Cholula, Puebla, C.P. 72750</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Maquila y fábrica de ropa y uniformes deportivos en paquete completo, con sublimado, estampado y transfer; empresa IMMEX.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de exportación de confección (IMMEX, SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>Empresa IMMEX de ropa deportiva: 50,000 prendas/semana en confección y 20,000 en sublimado digital; maquila de exportación.</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.directoriodefabricas.com/mexico/proveedores-de-ropa-directo-de-fabrica-en-puebla.html</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr"/>
       <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.directoriodefabricas.com/mexico/proveedores-de-ropa-directo-de-fabrica-en-puebla.html</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr"/>
+      <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1503,33 +1915,53 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>Km. 8 Antigua Carretera a Tlaxcala, Vía Fábricas, Colonia Guadalupe Caleras, C.P. 72100, Puebla, Pue.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Fábrica textil poblana que ofrece productos y servicios textiles, incluida maquila de estampado e impresión con tintas reactivas.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>Maquila de estampado e impresión con tintas reactivas para la industria textil poblana; podría comprar pastas base agua.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>https://www.lamaria.com.mx/</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>https://www.lamaria.com.mx/maquiladoras-textiles-en-puebla/</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr"/>
+      <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1554,33 +1986,53 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
+          <t>3 Sur 1910-3, C.P. 72500, Puebla, Pue.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de impresión en serigrafía y tampografía en equipos automatizados (Reflex), incluida producción para campañas.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>Maquila de serigrafía para grandes volúmenes (campañas políticas).</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>https://serigrafiapuebla.com/</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>https://serigrafiapuebla.com/</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr"/>
-      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr"/>
+      <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1605,29 +2057,53 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
+          <t>Blvd. Aeropuerto No. 425 D, Fracciones del Predio Sta. Julia de Jerez, C.P. 37290, León, Guanajuato (Inter Tenis, S.A. de C.V.)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Grupo mexicano de calzado y ropa deportiva (marca Charly) que diseña, fabrica y comercializa calzado, jerseys de clubes y ropa deportiva.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>Marca de León que viste a varios clubes de Liga MX (León, Pachuca, Atlas, Santos, Querétaro); produce jerseys y licencias en volumen.</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>https://lasillarota.com/guanajuato/2021/9/15/nueve-equipos-de-primera-division-usan-playeras-fabricadas-en-guanajuato-262317.html</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr"/>
       <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>https://lasillarota.com/guanajuato/2021/9/15/nueve-equipos-de-primera-division-usan-playeras-fabricadas-en-guanajuato-262317.html</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr"/>
+      <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Grupo Charly es principalmente de calzado; los jerseys podrían maquilarse fuera (Grupo Martex menciona a Charly como cliente). Confirmar si estampa en planta propia.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1652,33 +2128,53 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
+          <t>Palestina #102, Col. San Felipe de Jesús, León, Guanajuato</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Impresión textil en serigrafía (plastisol, base agua, descarga, especiales) y DTF para marcas, uniformes y promocionales.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>Más de 20 años en impresión textil: serigrafía (incluye descarga a 4 tintas) y DTF. Podría pasar a un híbrido.</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>https://galandserigrafia.com/</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>https://galandserigrafia.com/</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr"/>
+      <c r="P24" s="3" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1703,33 +2199,57 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
+          <t>Boulevard Uriangato #342, Col. La Joyita, C.P. 38983, Uriangato, Guanajuato</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de tejido de punto (suéteres, cardigans, vestidos, tops) con diseño y producción en un solo lugar, 2,000 piezas por semana.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Tejido de punto y confección (SCIAN 3132/315)</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>Maquila de tejido de punto con capacidad de 2,000 piezas/semana; diseño y producción en un mismo lugar.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr">
         <is>
           <t>https://grupotextilinma.com/</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>https://grupotextilinma.com/</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="3" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr"/>
+      <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Hace tejido de punto en galga fina (suéteres); no se menciona estampado. La dirección publicada está en Uriangato, no en Moroleón.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1754,33 +2274,53 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
+          <t>Mariano Talavera #312, Guanajuato, México</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Marca guanajuatense de calzado y ropa deportiva que vende jerseys de clubes, ropa y uniformes de equipo.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>Marca guanajuatense de ropa deportiva que viste a clubes de Liga MX (Necaxa, Atlético San Luis, Mazatlán) y vende uniformes de equipo.</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>https://pirma.com.mx/</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>https://lasillarota.com/guanajuato/2021/9/15/nueve-equipos-de-primera-division-usan-playeras-fabricadas-en-guanajuato-262317.html</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="3" t="inlineStr"/>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr"/>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1805,37 +2345,57 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
+          <t>Calle Pedro Guzmán no. 26, Col. Centro, C.P. 38800, Moroleón, Gto. (sucursal Moroleón)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Grupo textil de Moroleón que fabrica y estampa playeras (publicitarias y tipo polo), cobijas, banderas, gorras y uniformes.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Grupo textil de Moroleón con área de estampado textil; abastece al corredor Moroleón-Uriangato.</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>https://tejidosgaytan.com.mx/</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>ventas@tejidosgaytan.com.mx / 445 458 1888</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>https://tejidosgaytan.com.mx/grupo-textil/estampado-textil/</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
-      <c r="M27" s="3" t="inlineStr"/>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr"/>
+      <c r="P27" s="3" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1860,33 +2420,53 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
+          <t>Privada Arnulfo Garza No. 109, Col. Rincón de Santa María, Monterrey, N.L., C.P. 64650</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica uniformes corporativos y playeras tipo polo desde 2002 (marca Sparviero), con bordado, serigrafía y transfer.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>Polos y uniformes corporativos (Dry &amp; Cool); su planta integra bordado industrial, serigrafía y transfer.</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>https://www.sparviero.com.mx/</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-playeras-en-mexico.php</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr"/>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr"/>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr"/>
+      <c r="P28" s="3" t="inlineStr"/>
+      <c r="Q28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1911,33 +2491,53 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
+          <t>José Treviño 1222, Centro, C.P. 64000, Monterrey, N.L.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de ropa deportiva en paquete completo para marcas, con sublimación digital, DTF y DTG.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>Maquila de paquete completo para marcas, con sublimación digital, DTF y DTG; ya invierte en digital.</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr">
         <is>
           <t>https://maquiladeropadeportiva.com/</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr"/>
+      <c r="P29" s="3" t="inlineStr"/>
+      <c r="Q29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1962,33 +2562,53 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
+          <t>Pájaros Azules 4306, Col. Nuevo Almaguer, Guadalupe, N.L., C.P. 67183</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica y distribuye uniformes industriales y escolares con bordado, serigrafía y sublimación en planta propia (Vázquez Villarreal – VVF).</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>Fábrica de uniformes industriales y escolares con bordado, serigrafía y sublimación en planta propia; vende en México y EE.UU.</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>https://vvfdistribucion.mx/</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>https://vvfdistribucion.mx/uniformes/</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr"/>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2013,33 +2633,53 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
+          <t>Calle 63 No 453-A por 48 y 50, Centro, C.P. 97000 (Mérida, Yuc.)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Empresa integrada de tejido de punto que produce hilos, telas y playeras, con serigrafía y transfer propios.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Tejido de punto y confección (SCIAN 3132/315)</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>Integrado: hilos, telas y playeras, con serigrafía y transfer propios.</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>http://www.grupowabi.com/</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>http://www.grupowabi.com/Playeras.html</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="3" t="inlineStr"/>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr"/>
+      <c r="P31" s="3" t="inlineStr"/>
+      <c r="Q31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2064,33 +2704,53 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
+          <t>Calle 65 #365 entre 40 y 42, Col. Centro (Matriz, Mérida, Yuc.)</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica, personaliza y suministra uniformes, playeras, polos y promocionales, con lavado y teñido, bordado y serigrafía.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>Uniformes con áreas propias de teñido, estampado, sublimado y bordado; surte a cadenas comerciales y campañas políticas.</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>https://www.yoyos.mx/</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-uniformes-en-mexico.html</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O32" s="3" t="inlineStr"/>
+      <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2115,33 +2775,53 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
+          <t>Colinas de Veracruz, Colinas de San Pablo, C.P. 76125, Santiago de Querétaro, Querétaro (sin número publicado)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica uniformes (empresariales, escolares, industriales y deportivos) con bordado, sublimación, DTF y serigrafía, y ofrece publicidad y promocionales.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes (SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>Fabricación de uniformes con serigrafía, impresión digital y bordado; cercano a TID.</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="K33" s="3" t="inlineStr">
         <is>
           <t>https://www.grupojasedi.com/</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr">
         <is>
           <t>https://www.grupojasedi.com/</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr"/>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr"/>
+      <c r="P33" s="3" t="inlineStr"/>
+      <c r="Q33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2166,29 +2846,49 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
+          <t>Calzada Gómez Morín S/N, Col. Lajat, Torreón, Coahuila</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Planta de confección de exportación en Torreón (también TBG Apparel / Delta Apparel) registrada en Open Supply Hub con estampado, teñido, lavandería y corte y costura para Levi Strauss.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de exportación de confección (IMMEX, SCIAN 315)</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
           <t>Maquiladora de exportación</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>Planta de exportación (proveedor de Levi Strauss) con procesos de estampado (printing), lavandería y confección.</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>https://opensupplyhub.org/facilities/MX2021221QDMF7X</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>https://opensupplyhub.org/facilities/MX2021221QDMF7X</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr"/>
+      <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2213,33 +2913,53 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
+          <t>No publicada</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Taller de maquila de serigrafía textil y DTF en Aguascalientes para tiendas, eventos y campañas políticas (sitio solo indica 'Aguascalientes, México').</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Estampado y serigrafía textil (acabado, SCIAN 3133)</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
           <t>Estampador industrial</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>Taller de maquila de serigrafía textil con más de 15 años (serigrafía y DTF).</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="K35" s="3" t="inlineStr">
         <is>
           <t>https://salazarcervantes.click/</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr">
         <is>
           <t>https://salazarcervantes.click/</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr"/>
-      <c r="M35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O35" s="3" t="inlineStr"/>
+      <c r="P35" s="3" t="inlineStr"/>
+      <c r="Q35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2262,35 +2982,39 @@
           <t>Naucalpan de Juárez, Edo. Méx.</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Ropa deportiva y uniformes escolares con marca propia SWING.</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>https://ropadeportivaswing.com/</t>
-        </is>
-      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
+          <t>Fabricante de ropa deportiva/uniformes</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Ropa deportiva y uniformes escolares con marca propia SWING.</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>https://ropadeportivaswing.com/</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr"/>
+      <c r="P36" s="3" t="inlineStr"/>
+      <c r="Q36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2313,35 +3037,39 @@
           <t>Ciudad de México (Vallejo)</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>Marca de ropa deportiva de gama alta con red nacional de tiendas; posible uso de estampado y efectos especiales.</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>https://highimpact.com.mx/</t>
-        </is>
-      </c>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Marca de ropa deportiva de gama alta con red nacional de tiendas; posible uso de estampado y efectos especiales.</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>https://highimpact.com.mx/</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-deportiva-en-mexico.html</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K37" s="3" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr"/>
-      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr"/>
+      <c r="P37" s="3" t="inlineStr"/>
+      <c r="Q37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2364,35 +3092,39 @@
           <t>Naucalpan de Juárez, Edo. Méx.</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Grupo textil integrado (hilo, tela, teñido y confección) que vende sudaderas, joggers y playeras al mayoreo; posible cliente de consumibles y estampado.</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>https://optimamayoreo.com.mx/</t>
-        </is>
-      </c>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Grupo textil integrado (hilo, tela, teñido y confección) que vende sudaderas, joggers y playeras al mayoreo; posible cliente de consumibles y estampado.</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>https://optimamayoreo.com.mx/</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-sudaderas-en-mexico.php</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O38" s="3" t="inlineStr"/>
+      <c r="P38" s="3" t="inlineStr"/>
+      <c r="Q38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2415,31 +3147,35 @@
           <t>Guadalajara, Jal.</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>Maquila de activewear, rashguards y marcas de terceros, con sublimación y bordado; distribución nacional e internacional.</t>
-        </is>
-      </c>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-guadalajara-jalisco.html</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Maquila de activewear, rashguards y marcas de terceros, con sublimación y bordado; distribución nacional e internacional.</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr"/>
       <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-guadalajara-jalisco.html</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr"/>
+      <c r="P39" s="3" t="inlineStr"/>
+      <c r="Q39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2462,35 +3198,39 @@
           <t>Guadalajara, Jal.</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>Maquila de ropa deportiva sublimada (10,000 piezas/mes) con exportación a Europa y Norteamérica.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/gigafitness.mx</t>
-        </is>
-      </c>
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr"/>
+      <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
+          <t>Maquiladora de exportación</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de ropa deportiva sublimada (10,000 piezas/mes) con exportación a Europa y Norteamérica.</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/gigafitness.mx</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-guadalajara-jalisco.html</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O40" s="3" t="inlineStr"/>
+      <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2513,35 +3253,39 @@
           <t>Zapotlanejo, Jal.</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Empresa textil de moda en Zapotlanejo, un clúster de más de 400 talleres. Sirve como puerta de entrada al clúster; su tamaño está por verificar.</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/textilsurtimoda/</t>
-        </is>
-      </c>
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Empresa textil de moda en Zapotlanejo, un clúster de más de 400 talleres. Sirve como puerta de entrada al clúster; su tamaño está por verificar.</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
           <t>https://www.instagram.com/textilsurtimoda/</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/textilsurtimoda/</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr"/>
+      <c r="P41" s="3" t="inlineStr"/>
+      <c r="Q41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2564,35 +3308,39 @@
           <t>Guadalajara, Jal.</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>Uniformes corporativos y promocionales (líneas ejecutiva, promocional, casual e industrial).</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>https://www.topuniformes.mx/</t>
-        </is>
-      </c>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
+          <t>Fabricante de ropa deportiva/uniformes</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Uniformes corporativos y promocionales (líneas ejecutiva, promocional, casual e industrial).</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.topuniformes.mx/</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-uniformes-en-mexico.html</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr"/>
-      <c r="M42" s="3" t="inlineStr"/>
+      <c r="N42" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O42" s="3" t="inlineStr"/>
+      <c r="P42" s="3" t="inlineStr"/>
+      <c r="Q42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2615,35 +3363,39 @@
           <t>Contla, Tlax.</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante tlaxcalteca de sudaderas y chamarras con fibras recicladas; podría comprar tintas base agua o ecológicas.</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>https://www.amltextil.com/</t>
-        </is>
-      </c>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Fabricante tlaxcalteca de sudaderas y chamarras con fibras recicladas; podría comprar tintas base agua o ecológicas.</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
           <t>https://www.amltextil.com/</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K43" s="3" t="inlineStr"/>
       <c r="L43" s="3" t="inlineStr"/>
-      <c r="M43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amltextil.com/</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr"/>
+      <c r="P43" s="3" t="inlineStr"/>
+      <c r="Q43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2666,35 +3418,39 @@
           <t>Tlaxcala (zona Puebla-Tlaxcala)</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Promocionales</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de playeras de varios tejidos con servicio de estampado. Ubicación exacta y tamaño por verificar.</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/ConfeccionesRomers/</t>
-        </is>
-      </c>
+      <c r="E44" s="3" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr"/>
+      <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
+          <t>Promocionales</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Fabricante de playeras de varios tejidos con servicio de estampado. Ubicación exacta y tamaño por verificar.</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ConfeccionesRomers/</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
           <t>https://www.facebook.com/ConfeccionesRomers/posts/en-confecciones-romers-tenemos-variedad-en-playeras-para-tu-negocio-cont%C3%A1ctanos-/1451052420400737/</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr"/>
-      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="inlineStr"/>
+      <c r="P44" s="3" t="inlineStr"/>
+      <c r="Q44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2717,31 +3473,35 @@
           <t>San Andrés Cholula, Pue.</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Maquila de paquete completo de ropa deportiva y seamless, con 400 máquinas de costura y exportación. Decoración por confirmar.</t>
-        </is>
-      </c>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>https://www.directoriodefabricas.com/mexico/proveedores-de-ropa-directo-de-fabrica-en-puebla.html</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Maquila de paquete completo de ropa deportiva y seamless, con 400 máquinas de costura y exportación. Decoración por confirmar.</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr"/>
       <c r="L45" s="3" t="inlineStr"/>
-      <c r="M45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.directoriodefabricas.com/mexico/proveedores-de-ropa-directo-de-fabrica-en-puebla.html</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="inlineStr"/>
+      <c r="P45" s="3" t="inlineStr"/>
+      <c r="Q45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2764,35 +3524,39 @@
           <t>Puebla, Pue.</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Estampador industrial</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>Maquila de playeras deportivas con sublimación y vinil, con más de 15 años; podría sumar serigrafía o digital.</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>https://estampados.itipsa.com/</t>
-        </is>
-      </c>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr">
         <is>
+          <t>Estampador industrial</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Maquila de playeras deportivas con sublimación y vinil, con más de 15 años; podría sumar serigrafía o digital.</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
           <t>https://estampados.itipsa.com/</t>
         </is>
       </c>
-      <c r="J46" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K46" s="3" t="inlineStr"/>
       <c r="L46" s="3" t="inlineStr"/>
-      <c r="M46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>https://estampados.itipsa.com/</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr"/>
+      <c r="P46" s="3" t="inlineStr"/>
+      <c r="Q46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2815,35 +3579,39 @@
           <t>León, Gto.</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Promocionales</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>Serigrafía para uniformes de trabajo, playeras de evento y promocionales en León y el Bajío.</t>
-        </is>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>https://bvuniformes.com/</t>
-        </is>
-      </c>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr">
         <is>
+          <t>Promocionales</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Serigrafía para uniformes de trabajo, playeras de evento y promocionales en León y el Bajío.</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>https://bvuniformes.com/</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
           <t>https://bvuniformes.com/decoracion/serigrafia</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr"/>
-      <c r="M47" s="3" t="inlineStr"/>
+      <c r="N47" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="inlineStr"/>
+      <c r="P47" s="3" t="inlineStr"/>
+      <c r="Q47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -2866,35 +3634,39 @@
           <t>Moroleón, Gto.</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de moda rápida que lanza unos 50 modelos nuevos por semana (sudaderas, blusas); vende en México y EE.UU.</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>https://modalandia.com/</t>
-        </is>
-      </c>
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr"/>
       <c r="H48" s="3" t="inlineStr"/>
       <c r="I48" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Fabricante de moda rápida que lanza unos 50 modelos nuevos por semana (sudaderas, blusas); vende en México y EE.UU.</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>https://modalandia.com/</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
           <t>https://www.directoriodefabricas.com/mexico/fabricantes-de-ropa-en-mexico.html</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
-      <c r="M48" s="3" t="inlineStr"/>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr"/>
+      <c r="P48" s="3" t="inlineStr"/>
+      <c r="Q48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2917,31 +3689,35 @@
           <t>León, Gto.</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Fábrica de uniformes deportivos personalizados para mayoristas.</t>
-        </is>
-      </c>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
       <c r="G49" s="3" t="inlineStr"/>
       <c r="H49" s="3" t="inlineStr"/>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/Luisintentodeyoutuber/videos/prosutex-f%C3%A1brica-de-ropa-deportiva-para-mayoristas-en-le%C3%B3n-guanajuato-m%C3%A9xico-fut/1935623337359257/</t>
+          <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Fábrica de uniformes deportivos personalizados para mayoristas.</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr"/>
       <c r="L49" s="3" t="inlineStr"/>
-      <c r="M49" s="3" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Luisintentodeyoutuber/videos/prosutex-f%C3%A1brica-de-ropa-deportiva-para-mayoristas-en-le%C3%B3n-guanajuato-m%C3%A9xico-fut/1935623337359257/</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="inlineStr"/>
+      <c r="P49" s="3" t="inlineStr"/>
+      <c r="Q49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -2964,35 +3740,39 @@
           <t>Monterrey, N.L.</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>Promocionales</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>Fabrica sudaderas, playeras dry fit y uniformes con bordado, serigrafía y sublimación.</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>https://www.camisetasmonterrey.com.mx/</t>
-        </is>
-      </c>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="3" t="inlineStr"/>
       <c r="I50" s="3" t="inlineStr">
         <is>
+          <t>Promocionales</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Fabrica sudaderas, playeras dry fit y uniformes con bordado, serigrafía y sublimación.</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
           <t>https://www.camisetasmonterrey.com.mx/</t>
         </is>
       </c>
-      <c r="J50" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K50" s="3" t="inlineStr"/>
       <c r="L50" s="3" t="inlineStr"/>
-      <c r="M50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>https://www.camisetasmonterrey.com.mx/</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O50" s="3" t="inlineStr"/>
+      <c r="P50" s="3" t="inlineStr"/>
+      <c r="Q50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -3015,31 +3795,35 @@
           <t>Motul, Yuc.</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>Unos 1,800 empleados; exporta ropa casual, de punto y outerwear a EE.UU. (L.L. Bean, entre otros). Decoración por confirmar.</t>
-        </is>
-      </c>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="3" t="inlineStr"/>
       <c r="H51" s="3" t="inlineStr"/>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Unos 1,800 empleados; exporta ropa casual, de punto y outerwear a EE.UU. (L.L. Bean, entre otros). Decoración por confirmar.</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr"/>
       <c r="L51" s="3" t="inlineStr"/>
-      <c r="M51" s="3" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O51" s="3" t="inlineStr"/>
+      <c r="P51" s="3" t="inlineStr"/>
+      <c r="Q51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -3062,31 +3846,35 @@
           <t>Yucatán</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>Exportador de ropa con envíos constantes a EE.UU. por Progreso. Tamaño y decoración por confirmar.</t>
-        </is>
-      </c>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr"/>
       <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="3" t="inlineStr"/>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Exportador de ropa con envíos constantes a EE.UU. por Progreso. Tamaño y decoración por confirmar.</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr"/>
       <c r="L52" s="3" t="inlineStr"/>
-      <c r="M52" s="3" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr"/>
+      <c r="P52" s="3" t="inlineStr"/>
+      <c r="Q52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -3109,35 +3897,39 @@
           <t>Querétaro, Qro.</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Promocionales</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Fabricación propia de playeras con bordado, serigrafía y DTF para empresas.</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>https://www.playerasgarvel.com/</t>
-        </is>
-      </c>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="3" t="inlineStr"/>
       <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
+          <t>Promocionales</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Fabricación propia de playeras con bordado, serigrafía y DTF para empresas.</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
           <t>https://www.playerasgarvel.com/</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr"/>
       <c r="L53" s="3" t="inlineStr"/>
-      <c r="M53" s="3" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.playerasgarvel.com/</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="inlineStr"/>
+      <c r="P53" s="3" t="inlineStr"/>
+      <c r="Q53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -3160,35 +3952,39 @@
           <t>Querétaro, Qro.</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de uniformes con serigrafía y sublimación (uniformes deportivos).</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>https://www.uniformesuniverso.com.mx/</t>
-        </is>
-      </c>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr"/>
       <c r="I54" s="3" t="inlineStr">
         <is>
+          <t>Fabricante de ropa deportiva/uniformes</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Fabricante de uniformes con serigrafía y sublimación (uniformes deportivos).</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
           <t>https://www.uniformesuniverso.com.mx/</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr"/>
       <c r="L54" s="3" t="inlineStr"/>
-      <c r="M54" s="3" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.uniformesuniverso.com.mx/</t>
+        </is>
+      </c>
+      <c r="N54" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="inlineStr"/>
+      <c r="P54" s="3" t="inlineStr"/>
+      <c r="Q54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3211,39 +4007,43 @@
           <t>Querétaro, Qro.</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="3" t="inlineStr"/>
+      <c r="H55" s="3" t="inlineStr"/>
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>Fabricante de ropa deportiva/uniformes</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="J55" s="3" t="inlineStr">
         <is>
           <t>Uniformes y estampado de playeras en serigrafía y vinil textil.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="K55" s="3" t="inlineStr">
         <is>
           <t>https://www.uniformesenqueretaro.com.mx/</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="L55" s="3" t="inlineStr">
         <is>
           <t>(442) 213 28 86</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="M55" s="3" t="inlineStr">
         <is>
           <t>https://www.uniformesenqueretaro.com.mx/estampado-textil-queretaro.php</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr"/>
-      <c r="L55" s="3" t="inlineStr"/>
-      <c r="M55" s="3" t="inlineStr"/>
+      <c r="N55" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O55" s="3" t="inlineStr"/>
+      <c r="P55" s="3" t="inlineStr"/>
+      <c r="Q55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -3266,31 +4066,35 @@
           <t>Gómez Palacio, Dgo.</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de prendas desde 2008 para mercado nacional e internacional. Decoración por confirmar.</t>
-        </is>
-      </c>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr"/>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>https://www.sourceready.com/supplier/list/best-mexican-clothing-manufacturers-mx</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Fabricante de prendas desde 2008 para mercado nacional e internacional. Decoración por confirmar.</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr"/>
       <c r="L56" s="3" t="inlineStr"/>
-      <c r="M56" s="3" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sourceready.com/supplier/list/best-mexican-clothing-manufacturers-mx</t>
+        </is>
+      </c>
+      <c r="N56" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="inlineStr"/>
+      <c r="P56" s="3" t="inlineStr"/>
+      <c r="Q56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3313,31 +4117,35 @@
           <t>Gómez Palacio, Dgo.</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>Maquiladora de exportación</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>Unas 500,000 unidades/mes para marcas de EE.UU.; principalmente mezclilla, con bordado. Encaje limitado (consumibles o estampado de bolsillos).</t>
-        </is>
-      </c>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr"/>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+          <t>Maquiladora de exportación</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>Por contactar</t>
+          <t>Unas 500,000 unidades/mes para marcas de EE.UU.; principalmente mezclilla, con bordado. Encaje limitado (consumibles o estampado de bolsillos).</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr"/>
       <c r="L57" s="3" t="inlineStr"/>
-      <c r="M57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cosmosourcing.com/blog/clothing-manufacturers-mexico</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="inlineStr"/>
+      <c r="P57" s="3" t="inlineStr"/>
+      <c r="Q57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -3360,35 +4168,39 @@
           <t>Torreón / La Laguna</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Uniformes con sublimado, bordado y serigrafía en La Laguna.</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>https://www.xpresionuniformesmx.com/</t>
-        </is>
-      </c>
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr"/>
+      <c r="G58" s="3" t="inlineStr"/>
       <c r="H58" s="3" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
+          <t>Fabricante de ropa deportiva/uniformes</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Uniformes con sublimado, bordado y serigrafía en La Laguna.</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
           <t>https://www.xpresionuniformesmx.com/</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr"/>
       <c r="L58" s="3" t="inlineStr"/>
-      <c r="M58" s="3" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.xpresionuniformesmx.com/</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr"/>
+      <c r="P58" s="3" t="inlineStr"/>
+      <c r="Q58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3411,35 +4223,39 @@
           <t>Aguascalientes, Ags.</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Marca de moda</t>
-        </is>
-      </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>Se anuncia como la fábrica de blanks (playeras oversize, sudaderas) más grande de Aguascalientes; podría integrar estampado.</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/reel/DOXNfMnjCNu/</t>
-        </is>
-      </c>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="3" t="inlineStr"/>
       <c r="H59" s="3" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
+          <t>Marca de moda</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Se anuncia como la fábrica de blanks (playeras oversize, sudaderas) más grande de Aguascalientes; podría integrar estampado.</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
           <t>https://www.instagram.com/reel/DOXNfMnjCNu/</t>
         </is>
       </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K59" s="3" t="inlineStr"/>
       <c r="L59" s="3" t="inlineStr"/>
-      <c r="M59" s="3" t="inlineStr"/>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DOXNfMnjCNu/</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="inlineStr"/>
+      <c r="P59" s="3" t="inlineStr"/>
+      <c r="Q59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3462,35 +4278,39 @@
           <t>Aguascalientes, Ags.</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>Estampador industrial</t>
-        </is>
-      </c>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>Fábrica de telas con estampado e impresión digital de tela y corte láser; posible comprador de consumibles.</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>https://www.satinexport.com/</t>
-        </is>
-      </c>
+      <c r="E60" s="3" t="inlineStr"/>
+      <c r="F60" s="3" t="inlineStr"/>
+      <c r="G60" s="3" t="inlineStr"/>
       <c r="H60" s="3" t="inlineStr"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
+          <t>Estampador industrial</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Fábrica de telas con estampado e impresión digital de tela y corte láser; posible comprador de consumibles.</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
           <t>https://www.satinexport.com/</t>
         </is>
       </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K60" s="3" t="inlineStr"/>
       <c r="L60" s="3" t="inlineStr"/>
-      <c r="M60" s="3" t="inlineStr"/>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>https://www.satinexport.com/</t>
+        </is>
+      </c>
+      <c r="N60" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O60" s="3" t="inlineStr"/>
+      <c r="P60" s="3" t="inlineStr"/>
+      <c r="Q60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -3513,40 +4333,44 @@
           <t>Aguascalientes, Ags.</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>Fabricante de ropa deportiva/uniformes</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>Fabricación de uniformes industriales, escolares y deportivos; playeras.</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>https://www.uniformesbreceda.com/</t>
-        </is>
-      </c>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr"/>
       <c r="H61" s="3" t="inlineStr"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
+          <t>Fabricante de ropa deportiva/uniformes</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Fabricación de uniformes industriales, escolares y deportivos; playeras.</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
           <t>https://www.uniformesbreceda.com/</t>
         </is>
       </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>Por contactar</t>
-        </is>
-      </c>
-      <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr"/>
-      <c r="M61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.uniformesbreceda.com/</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>Por contactar</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr"/>
+      <c r="P61" s="3" t="inlineStr"/>
+      <c r="Q61" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M61"/>
+  <autoFilter ref="A1:Q61"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Por contactar,Contactado,Visita agendada,Demo,Cotización,Ganado,Perdido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>